<commit_message>
feat(analysis): Implement longitudinal SVI model & 2030 forecast
- Added Master Profile dataset (2010-2024) with robust error handling
- Implemented Social Vulnerability Index (SVI) ranking logic
- Added K-Means Clustering to identify 'Risk Profiles'
- Developed 'Evacuation Crisis' and 'Blight/Abandonment' indices
- Implemented Linear Regression model for 2030 SVI forecasting
- Generated final Executive Synthesis for dashboard integration
</commit_message>
<xml_diff>
--- a/data/crime/PR_Crime_Summary_2010_2025.xlsx
+++ b/data/crime/PR_Crime_Summary_2010_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/venettov/Documents/Capstone/CAPSTONE_DATA_SCIENCE_RIVERARUIZ/data/crime/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D851435F-3A25-C442-8F95-4F808BE47722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F195FA5-54A2-BB45-B7AC-5FBE4D1C3F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{43E4E03C-6A79-7E4D-A8F1-AF00C31A2DE9}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" activeTab="16" xr2:uid="{43E4E03C-6A79-7E4D-A8F1-AF00C31A2DE9}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="224">
   <si>
     <t>Totales</t>
   </si>
@@ -1093,6 +1093,9 @@
   <si>
     <t>Se debe incluir el llevarse un vehículo sin permiso del dueño para realizar paseos alocados.</t>
   </si>
+  <si>
+    <t>Data from: Statistics_Institute_of_Puerto_Rico</t>
+  </si>
 </sst>
 </file>
 
@@ -1290,27 +1293,27 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1659,7 +1662,7 @@
     <col min="7" max="7" width="8.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.5" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.5" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -6267,7 +6270,7 @@
         <v>895</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>7943</v>
       </c>
     </row>
@@ -9018,7 +9021,7 @@
         <v>952</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>8368</v>
       </c>
     </row>
@@ -11489,7 +11492,7 @@
         <v>1140</v>
       </c>
       <c r="I66">
-        <f t="shared" ref="I66:I97" si="2">SUM(B66:H66)</f>
+        <f t="shared" ref="I66:I79" si="2">SUM(B66:H66)</f>
         <v>9567</v>
       </c>
     </row>
@@ -13916,7 +13919,7 @@
         <v>1283</v>
       </c>
       <c r="I66">
-        <f t="shared" ref="I66:I97" si="2">SUM(B66:H66)</f>
+        <f t="shared" ref="I66:I79" si="2">SUM(B66:H66)</f>
         <v>10464</v>
       </c>
     </row>
@@ -16859,35 +16862,35 @@
         <v>156</v>
       </c>
       <c r="B80" s="20">
-        <f>SUM(B2:B79)</f>
+        <f t="shared" ref="B80:I80" si="3">SUM(B2:B79)</f>
         <v>978</v>
       </c>
       <c r="C80" s="20">
-        <f>SUM(C2:C79)</f>
+        <f t="shared" si="3"/>
         <v>32</v>
       </c>
       <c r="D80" s="20">
-        <f>SUM(D2:D79)</f>
+        <f t="shared" si="3"/>
         <v>6298</v>
       </c>
       <c r="E80" s="20">
-        <f>SUM(E2:E79)</f>
+        <f t="shared" si="3"/>
         <v>2733</v>
       </c>
       <c r="F80" s="20">
-        <f>SUM(F2:F79)</f>
+        <f t="shared" si="3"/>
         <v>15287</v>
       </c>
       <c r="G80" s="20">
-        <f>SUM(G2:G79)</f>
+        <f t="shared" si="3"/>
         <v>30545</v>
       </c>
       <c r="H80" s="20">
-        <f>SUM(H2:H79)</f>
+        <f t="shared" si="3"/>
         <v>5847</v>
       </c>
       <c r="I80" s="20">
-        <f>SUM(I2:I79)</f>
+        <f t="shared" si="3"/>
         <v>61720</v>
       </c>
     </row>
@@ -19286,35 +19289,35 @@
         <v>156</v>
       </c>
       <c r="B80" s="20">
-        <f>SUM(B2:B79)</f>
+        <f t="shared" ref="B80:I80" si="3">SUM(B2:B79)</f>
         <v>1136</v>
       </c>
       <c r="C80" s="20">
-        <f>SUM(C2:C79)</f>
+        <f t="shared" si="3"/>
         <v>45</v>
       </c>
       <c r="D80" s="20">
-        <f>SUM(D2:D79)</f>
+        <f t="shared" si="3"/>
         <v>6465</v>
       </c>
       <c r="E80" s="20">
-        <f>SUM(E2:E79)</f>
+        <f t="shared" si="3"/>
         <v>2894</v>
       </c>
       <c r="F80" s="20">
-        <f>SUM(F2:F79)</f>
+        <f t="shared" si="3"/>
         <v>16591</v>
       </c>
       <c r="G80" s="20">
-        <f>SUM(G2:G79)</f>
+        <f t="shared" si="3"/>
         <v>29273</v>
       </c>
       <c r="H80" s="20">
-        <f>SUM(H2:H79)</f>
+        <f t="shared" si="3"/>
         <v>5853</v>
       </c>
       <c r="I80" s="20">
-        <f>SUM(I2:I79)</f>
+        <f t="shared" si="3"/>
         <v>62257</v>
       </c>
     </row>
@@ -21713,35 +21716,35 @@
         <v>156</v>
       </c>
       <c r="B80" s="20">
-        <f>SUM(B2:B79)</f>
+        <f t="shared" ref="B80:I80" si="3">SUM(B2:B79)</f>
         <v>983</v>
       </c>
       <c r="C80" s="20">
-        <f>SUM(C2:C79)</f>
+        <f t="shared" si="3"/>
         <v>39</v>
       </c>
       <c r="D80" s="20">
-        <f>SUM(D2:D79)</f>
+        <f t="shared" si="3"/>
         <v>6590</v>
       </c>
       <c r="E80" s="20">
-        <f>SUM(E2:E79)</f>
+        <f t="shared" si="3"/>
         <v>2753</v>
       </c>
       <c r="F80" s="20">
-        <f>SUM(F2:F79)</f>
+        <f t="shared" si="3"/>
         <v>17880</v>
       </c>
       <c r="G80" s="20">
-        <f>SUM(G2:G79)</f>
+        <f t="shared" si="3"/>
         <v>27182</v>
       </c>
       <c r="H80" s="20">
-        <f>SUM(H2:H79)</f>
+        <f t="shared" si="3"/>
         <v>6811</v>
       </c>
       <c r="I80" s="20">
-        <f>SUM(I2:I79)</f>
+        <f t="shared" si="3"/>
         <v>62238</v>
       </c>
     </row>
@@ -21869,7 +21872,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77629FE4-0AAF-4F45-8D35-1C3005808586}">
-  <dimension ref="A2:J46"/>
+  <dimension ref="A2:J49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" style="22" customWidth="1"/>
@@ -22195,12 +22198,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="32" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
       <c r="E2" s="24"/>
       <c r="F2" s="24"/>
       <c r="G2" s="24"/>
@@ -22209,341 +22212,341 @@
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="24"/>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="32" t="s">
         <v>193</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="32" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="25"/>
-      <c r="B7" s="23" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="32" t="s">
         <v>195</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="25"/>
-      <c r="B8" s="26" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="25"/>
-      <c r="B9" s="26" t="s">
+      <c r="A9" s="23"/>
+      <c r="B9" s="30" t="s">
         <v>197</v>
       </c>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
     </row>
     <row r="10" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="24"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="23" t="s">
         <v>198</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="28"/>
-      <c r="B12" s="25" t="s">
+      <c r="A12" s="25"/>
+      <c r="B12" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="25"/>
-      <c r="B13" s="28" t="s">
+      <c r="A13" s="23"/>
+      <c r="B13" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="25"/>
-      <c r="B14" s="28" t="s">
+      <c r="A14" s="23"/>
+      <c r="B14" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="27" t="s">
         <v>202</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A16" s="24"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="25"/>
-      <c r="B18" s="23" t="s">
+      <c r="A18" s="23"/>
+      <c r="B18" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="25"/>
-      <c r="B19" s="26" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="30" t="s">
         <v>205</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="25"/>
-      <c r="B20" s="26" t="s">
+      <c r="A20" s="23"/>
+      <c r="B20" s="30" t="s">
         <v>206</v>
       </c>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
     </row>
     <row r="21" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" s="24"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
     </row>
     <row r="22" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A22" s="24"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="25"/>
-      <c r="B24" s="25" t="s">
+      <c r="A24" s="23"/>
+      <c r="B24" s="23" t="s">
         <v>208</v>
       </c>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="25"/>
-      <c r="B25" s="28" t="s">
+      <c r="A25" s="23"/>
+      <c r="B25" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="25"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="25"/>
-      <c r="B26" s="28" t="s">
+      <c r="A26" s="23"/>
+      <c r="B26" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="27"/>
     </row>
     <row r="28" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A28" s="24"/>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
     </row>
     <row r="29" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A29" s="24"/>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
     </row>
     <row r="30" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A30" s="30" t="s">
+      <c r="A30" s="28" t="s">
         <v>212</v>
       </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
       <c r="E30" s="24"/>
       <c r="F30" s="24"/>
       <c r="G30" s="24"/>
@@ -22552,36 +22555,36 @@
     </row>
     <row r="31" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A31" s="24"/>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="34" t="s">
         <v>213</v>
       </c>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
     </row>
     <row r="32" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A32" s="24"/>
-      <c r="B32" s="32" t="s">
+      <c r="B32" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
-      <c r="I32" s="32"/>
-      <c r="J32" s="32"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="35"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="35"/>
     </row>
     <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A33" s="24"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="33"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="24"/>
       <c r="E33" s="24"/>
       <c r="F33" s="24"/>
@@ -22590,11 +22593,11 @@
       <c r="I33" s="24"/>
     </row>
     <row r="35" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A35" s="23" t="s">
+      <c r="A35" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B35" s="23"/>
-      <c r="C35" s="23"/>
+      <c r="B35" s="32"/>
+      <c r="C35" s="32"/>
       <c r="D35" s="24"/>
       <c r="E35" s="24"/>
       <c r="F35" s="24"/>
@@ -22604,48 +22607,48 @@
     </row>
     <row r="36" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A36" s="24"/>
-      <c r="B36" s="34" t="s">
+      <c r="B36" s="33" t="s">
         <v>216</v>
       </c>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
-      <c r="J36" s="34"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="33"/>
     </row>
     <row r="37" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A37" s="24"/>
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="30" t="s">
         <v>217</v>
       </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
     </row>
     <row r="38" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
       <c r="F38" s="24"/>
       <c r="G38" s="24"/>
       <c r="H38" s="24"/>
       <c r="I38" s="24"/>
     </row>
     <row r="40" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A40" s="23" t="s">
+      <c r="A40" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B40" s="23"/>
+      <c r="B40" s="32"/>
       <c r="C40" s="24"/>
       <c r="D40" s="24"/>
       <c r="E40" s="24"/>
@@ -22656,23 +22659,23 @@
     </row>
     <row r="41" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="32" t="s">
         <v>219</v>
       </c>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="23"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
       <c r="H41" s="24"/>
       <c r="I41" s="24"/>
     </row>
     <row r="42" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A42" s="24"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
       <c r="F42" s="24"/>
       <c r="G42" s="24"/>
       <c r="H42" s="24"/>
@@ -22680,59 +22683,76 @@
     </row>
     <row r="43" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A43" s="24"/>
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="30" t="s">
         <v>220</v>
       </c>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="26"/>
-      <c r="J43" s="26"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="30"/>
+      <c r="J43" s="30"/>
     </row>
     <row r="44" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A44" s="24"/>
-      <c r="B44" s="26" t="s">
+      <c r="B44" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="C44" s="26"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="26"/>
-      <c r="I44" s="26"/>
-      <c r="J44" s="26"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30"/>
+      <c r="E44" s="30"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="30"/>
+      <c r="I44" s="30"/>
+      <c r="J44" s="30"/>
     </row>
     <row r="45" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A45" s="24"/>
-      <c r="B45" s="26" t="s">
+      <c r="B45" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="26"/>
-      <c r="I45" s="26"/>
-      <c r="J45" s="26"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
+      <c r="E45" s="30"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
+      <c r="J45" s="30"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B46" s="35"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="35"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="31"/>
+      <c r="F46" s="31"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="31"/>
+      <c r="J46" s="31"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="22" t="s">
+        <v>223</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B9:J9"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B31:J31"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
     <mergeCell ref="B46:J46"/>
@@ -22742,18 +22762,6 @@
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="B41:G41"/>
     <mergeCell ref="B43:J43"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="B18:J18"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B20:J20"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B32:J32"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="B7:J7"/>
-    <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B9:J9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30795,7 +30803,7 @@
         <v>957</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>4851</v>
       </c>
     </row>
@@ -33842,7 +33850,7 @@
         <v>800</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>3897</v>
       </c>
     </row>
@@ -36764,7 +36772,7 @@
         <v>604</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>3751</v>
       </c>
     </row>
@@ -39686,7 +39694,7 @@
         <v>1133</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>6042</v>
       </c>
     </row>
@@ -42608,7 +42616,7 @@
         <v>1139</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J79" si="2">SUM(B66:I66)</f>
         <v>6837</v>
       </c>
     </row>
@@ -45200,7 +45208,7 @@
         <v>788</v>
       </c>
       <c r="J66">
-        <f t="shared" ref="J66:J97" si="2">SUM(B66:I66)</f>
+        <f t="shared" ref="J66:J80" si="2">SUM(B66:I66)</f>
         <v>6952</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize phase 1 notebook with crime data integration and perfect markdown structure
</commit_message>
<xml_diff>
--- a/data/crime/PR_Crime_Summary_2010_2025.xlsx
+++ b/data/crime/PR_Crime_Summary_2010_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/venettov/Documents/Capstone/CAPSTONE_DATA_SCIENCE_RIVERARUIZ/data/crime/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreruiz/Documents/Capstone/CAPSTONE_DATA_SCIENCE_RIVERARUIZ/data/crime/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F195FA5-54A2-BB45-B7AC-5FBE4D1C3F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A423A7-22E6-2F43-A760-2A72A5957F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" activeTab="16" xr2:uid="{43E4E03C-6A79-7E4D-A8F1-AF00C31A2DE9}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{43E4E03C-6A79-7E4D-A8F1-AF00C31A2DE9}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -1302,18 +1302,18 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22198,12 +22198,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
       <c r="E2" s="24"/>
       <c r="F2" s="24"/>
       <c r="G2" s="24"/>
@@ -22212,16 +22212,16 @@
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="24"/>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>193</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
@@ -22235,53 +22235,53 @@
       <c r="I4" s="23"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="23"/>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="23"/>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="32" t="s">
         <v>196</v>
       </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="23"/>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="32" t="s">
         <v>197</v>
       </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
     </row>
     <row r="10" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="24"/>
@@ -22374,10 +22374,10 @@
       <c r="I16" s="26"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="31" t="s">
         <v>203</v>
       </c>
-      <c r="B17" s="32"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="26"/>
       <c r="D17" s="26"/>
       <c r="E17" s="26"/>
@@ -22388,45 +22388,45 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="23"/>
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="31" t="s">
         <v>204</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="32"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="23"/>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="32" t="s">
         <v>205</v>
       </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="23"/>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
     </row>
     <row r="21" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" s="24"/>
@@ -22555,31 +22555,31 @@
     </row>
     <row r="31" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A31" s="24"/>
-      <c r="B31" s="34" t="s">
+      <c r="B31" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
     </row>
     <row r="32" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A32" s="24"/>
-      <c r="B32" s="35" t="s">
+      <c r="B32" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-      <c r="J32" s="35"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
     </row>
     <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A33" s="24"/>
@@ -22593,11 +22593,11 @@
       <c r="I33" s="24"/>
     </row>
     <row r="35" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A35" s="32" t="s">
+      <c r="A35" s="31" t="s">
         <v>215</v>
       </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
       <c r="D35" s="24"/>
       <c r="E35" s="24"/>
       <c r="F35" s="24"/>
@@ -22607,31 +22607,31 @@
     </row>
     <row r="36" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A36" s="24"/>
-      <c r="B36" s="33" t="s">
+      <c r="B36" s="35" t="s">
         <v>216</v>
       </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
-      <c r="J36" s="33"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="35"/>
+      <c r="F36" s="35"/>
+      <c r="G36" s="35"/>
+      <c r="H36" s="35"/>
+      <c r="I36" s="35"/>
+      <c r="J36" s="35"/>
     </row>
     <row r="37" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A37" s="24"/>
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="30"/>
-      <c r="I37" s="30"/>
-      <c r="J37" s="30"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="32"/>
+      <c r="J37" s="32"/>
     </row>
     <row r="38" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
@@ -22645,10 +22645,10 @@
       <c r="I38" s="24"/>
     </row>
     <row r="40" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A40" s="32" t="s">
+      <c r="A40" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="B40" s="32"/>
+      <c r="B40" s="31"/>
       <c r="C40" s="24"/>
       <c r="D40" s="24"/>
       <c r="E40" s="24"/>
@@ -22659,14 +22659,14 @@
     </row>
     <row r="41" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="32" t="s">
+      <c r="B41" s="31" t="s">
         <v>219</v>
       </c>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="31"/>
       <c r="H41" s="24"/>
       <c r="I41" s="24"/>
     </row>
@@ -22683,56 +22683,56 @@
     </row>
     <row r="43" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A43" s="24"/>
-      <c r="B43" s="30" t="s">
+      <c r="B43" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
-      <c r="I43" s="30"/>
-      <c r="J43" s="30"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="32"/>
     </row>
     <row r="44" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A44" s="24"/>
-      <c r="B44" s="30" t="s">
+      <c r="B44" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
-      <c r="I44" s="30"/>
-      <c r="J44" s="30"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
     </row>
     <row r="45" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A45" s="24"/>
-      <c r="B45" s="30" t="s">
+      <c r="B45" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
-      <c r="I45" s="30"/>
-      <c r="J45" s="30"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="32"/>
+      <c r="J45" s="32"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B46" s="31"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="31"/>
-      <c r="E46" s="31"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="31"/>
-      <c r="H46" s="31"/>
-      <c r="I46" s="31"/>
-      <c r="J46" s="31"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="34"/>
+      <c r="J46" s="34"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="22" t="s">
@@ -22741,6 +22741,15 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B44:J44"/>
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B46:J46"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B43:J43"/>
     <mergeCell ref="B32:J32"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B3:I3"/>
@@ -22753,15 +22762,6 @@
     <mergeCell ref="B19:J19"/>
     <mergeCell ref="B20:J20"/>
     <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="B45:J45"/>
-    <mergeCell ref="B46:J46"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B43:J43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>